<commit_message>
fix: remove workbook sheet protection to eliminate edit friction
The no-password protection on "2. Your Rubric" and "Decision Summary" still
prompted / blocked editing in Excel, which defeated the point of an editable
rubric. Removed sheet protection from both sheets entirely — nothing is locked,
nothing to unprotect. Replaced the "Review → Unprotect Sheet" guidance with
plain instructions: edit the criteria, weights, and scores; there are blank
rows for more criteria; the shaded cells calculate on their own. Formulas and
the Decision Summary pull-through are unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/Jaspen-Decision-Planning-Toolkit.xlsx
+++ b/frontend/public/Jaspen-Decision-Planning-Toolkit.xlsx
@@ -1189,7 +1189,7 @@
     <row r="5">
       <c r="A5" s="22" t="inlineStr">
         <is>
-          <t>This is a starting example — replace it with your own. Only the shaded cells calculate for you.</t>
+          <t>This is a starting example — edit everything to fit your decision. The shaded cells fill in on their own.</t>
         </is>
       </c>
     </row>
@@ -1424,15 +1424,14 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
+    <row r="22" ht="44" customHeight="1">
       <c r="A22" s="36" t="inlineStr">
         <is>
-          <t>The leading option is just the math on your inputs — a prompt for judgment, not the verdict. You'll pressure-test it next. To add criteria or restructure the sheet, choose Review → Unprotect Sheet (no password needed).</t>
+          <t>Make this rubric yours: rename the criteria, set the weights, and score your options. There are blank rows if you need more criteria. The shaded cells calculate on their own — you can leave those to the toolkit. The leading option is just the math on your inputs — a prompt for judgment, not the verdict. You'll pressure-test it next.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
   <mergeCells count="7">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B20:D20"/>
@@ -2032,7 +2031,6 @@
     <row r="19" ht="18" customHeight="1"/>
     <row r="20" ht="18" customHeight="1"/>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
   <mergeCells count="15">
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="A17:E20"/>

</xml_diff>